<commit_message>
Contains Standard deviation code
</commit_message>
<xml_diff>
--- a/RTP_Result_500M_86.xlsx
+++ b/RTP_Result_500M_86.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="45">
   <si>
     <t>Metric</t>
   </si>
@@ -35,7 +35,7 @@
     <t xml:space="preserve">Date created: </t>
   </si>
   <si>
-    <t>2026-October-24</t>
+    <t>2026-October-28</t>
   </si>
   <si>
     <t>Hit rate</t>
@@ -48,6 +48,12 @@
   </si>
   <si>
     <t>Hit Rate (%)</t>
+  </si>
+  <si>
+    <t>Variance</t>
+  </si>
+  <si>
+    <t>Std Dev</t>
   </si>
   <si>
     <t xml:space="preserve"> Spot 2 </t>
@@ -191,11 +197,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.046875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="14.6875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="7.19921875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="11.4296875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.4296875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -211,7 +220,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n" s="0">
-        <v>5.0E8</v>
+        <v>1.0E8</v>
       </c>
     </row>
     <row r="3">
@@ -219,7 +228,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>5.0E8</v>
+        <v>1.0E8</v>
       </c>
     </row>
     <row r="4">
@@ -227,7 +236,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>4.322245105E8</v>
+        <v>8.63942895E7</v>
       </c>
     </row>
     <row r="5">
@@ -235,7 +244,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>86.44</v>
+        <v>86.39</v>
       </c>
     </row>
     <row r="6">
@@ -275,131 +284,191 @@
       <c r="C12" t="s" s="1">
         <v>5</v>
       </c>
+      <c r="D12" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s" s="1">
+        <v>13</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>6.016</v>
+        <v>6.018</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>86.91</v>
+        <v>87.1</v>
+      </c>
+      <c r="D13" t="n" s="0">
+        <v>31.092198787790444</v>
+      </c>
+      <c r="E13" t="n" s="0">
+        <v>5.576037911258355</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>15.27</v>
+        <v>15.25</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>86.32</v>
+        <v>86.34</v>
+      </c>
+      <c r="D14" t="n" s="0">
+        <v>70.63652174961474</v>
+      </c>
+      <c r="E14" t="n" s="0">
+        <v>8.404553631788826</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>25.89</v>
+        <v>25.91</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>86.42</v>
+        <v>86.04</v>
+      </c>
+      <c r="D15" t="n" s="0">
+        <v>46.85321916425759</v>
+      </c>
+      <c r="E15" t="n" s="0">
+        <v>6.844941136653959</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>9.67</v>
+        <v>9.651</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>86.15</v>
+        <v>85.95</v>
+      </c>
+      <c r="D16" t="n" s="0">
+        <v>62.53194732582436</v>
+      </c>
+      <c r="E16" t="n" s="0">
+        <v>7.907714418580401</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>16.16</v>
+        <v>16.15</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>86.4</v>
+        <v>86.56</v>
+      </c>
+      <c r="D17" t="n" s="0">
+        <v>68.79407633264373</v>
+      </c>
+      <c r="E17" t="n" s="0">
+        <v>8.294219452886674</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18" t="n" s="0">
-        <v>23.65</v>
+        <v>23.68</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>86.49</v>
+        <v>86.63</v>
+      </c>
+      <c r="D18" t="n" s="0">
+        <v>68.52524663529859</v>
+      </c>
+      <c r="E18" t="n" s="0">
+        <v>8.277997743132007</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B19" t="n" s="0">
-        <v>10.24</v>
+        <v>10.23</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>86.72</v>
+        <v>86.39</v>
+      </c>
+      <c r="D19" t="n" s="0">
+        <v>163.74219007697567</v>
+      </c>
+      <c r="E19" t="n" s="0">
+        <v>12.796178729487005</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B20" t="n" s="0">
         <v>15.3</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>86.07</v>
+        <v>85.85</v>
+      </c>
+      <c r="D20" t="n" s="0">
+        <v>106.39355982438099</v>
+      </c>
+      <c r="E20" t="n" s="0">
+        <v>10.314725387734809</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B21" t="n" s="0">
         <v>21.21</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>86.53</v>
+        <v>86.69</v>
+      </c>
+      <c r="D21" t="n" s="0">
+        <v>51.41219377000365</v>
+      </c>
+      <c r="E21" t="n" s="0">
+        <v>7.170229687395213</v>
       </c>
     </row>
     <row r="22"/>
     <row r="23">
       <c r="A23" t="s" s="1">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B24" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B25" t="n" s="0">
-        <v>56.0277</v>
+        <v>56.0245</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B26" t="n" s="0">
         <v>37.96</v>
@@ -407,602 +476,602 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B27" t="n" s="0">
-        <v>6.016</v>
+        <v>6.018</v>
       </c>
     </row>
     <row r="28"/>
     <row r="29">
       <c r="A29" t="s" s="1">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B30" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B31" t="n" s="0">
-        <v>41.666</v>
+        <v>41.6747</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B32" t="n" s="0">
-        <v>43.0688</v>
+        <v>43.0708</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B33" t="n" s="0">
-        <v>13.8754</v>
+        <v>13.864</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B34" t="n" s="0">
-        <v>1.38971</v>
+        <v>1.39052</v>
       </c>
     </row>
     <row r="35"/>
     <row r="36">
       <c r="A36" t="s" s="1">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B37" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B38" t="n" s="0">
-        <v>30.8328</v>
+        <v>30.8581</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B39" t="n" s="0">
-        <v>43.2733</v>
+        <v>43.2328</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B40" t="n" s="0">
-        <v>21.2595</v>
+        <v>21.276</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B41" t="n" s="0">
-        <v>4.3277</v>
+        <v>4.32725</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B42" t="n" s="0">
-        <v>0.306702</v>
+        <v>0.305876</v>
       </c>
     </row>
     <row r="43"/>
     <row r="44">
       <c r="A44" t="s" s="1">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B45" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B46" t="n" s="0">
-        <v>22.7185</v>
+        <v>22.7342</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B47" t="n" s="0">
-        <v>40.563</v>
+        <v>40.5809</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B48" t="n" s="0">
-        <v>27.0481</v>
+        <v>27.0337</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B49" t="n" s="0">
-        <v>8.39569</v>
+        <v>8.38352</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B50" t="n" s="0">
-        <v>1.21027</v>
+        <v>1.20395</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B51" t="n" s="0">
-        <v>0.0644196</v>
+        <v>0.0637864</v>
       </c>
     </row>
     <row r="52"/>
     <row r="53">
       <c r="A53" t="s" s="1">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B54" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B55" t="n" s="0">
-        <v>16.6612</v>
+        <v>16.66</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B56" t="n" s="0">
-        <v>36.3489</v>
+        <v>36.3535</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B57" t="n" s="0">
-        <v>30.8323</v>
+        <v>30.8345</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B58" t="n" s="0">
-        <v>12.979</v>
+        <v>12.9778</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B59" t="n" s="0">
-        <v>2.85673</v>
+        <v>2.84951</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B60" t="n" s="0">
-        <v>0.308811</v>
+        <v>0.311675</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B61" t="n" s="0">
-        <v>0.013029</v>
+        <v>0.0129126</v>
       </c>
     </row>
     <row r="62"/>
     <row r="63">
       <c r="A63" t="s" s="1">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B64" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B65" t="n" s="0">
-        <v>12.1508</v>
+        <v>12.1617</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B66" t="n" s="0">
-        <v>31.5221</v>
+        <v>31.4915</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B67" t="n" s="0">
-        <v>32.673</v>
+        <v>32.6668</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B68" t="n" s="0">
-        <v>17.4933</v>
+        <v>17.515</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B69" t="n" s="0">
-        <v>5.22025</v>
+        <v>5.22051</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B70" t="n" s="0">
-        <v>0.864682</v>
+        <v>0.868166</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B71" t="n" s="0">
-        <v>0.0735555</v>
+        <v>0.074067</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B72" t="n" s="0">
-        <v>0.00242827</v>
+        <v>0.002251</v>
       </c>
     </row>
     <row r="73"/>
     <row r="74">
       <c r="A74" t="s" s="1">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B75" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B76" t="n" s="0">
-        <v>8.82287</v>
+        <v>8.81532</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B77" t="n" s="0">
-        <v>26.6467</v>
+        <v>26.6486</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B78" t="n" s="0">
-        <v>32.8133</v>
+        <v>32.8177</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B79" t="n" s="0">
-        <v>21.4785</v>
+        <v>21.4909</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B80" t="n" s="0">
-        <v>8.14976</v>
+        <v>8.14441</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B81" t="n" s="0">
-        <v>1.83252</v>
+        <v>1.83002</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B82" t="n" s="0">
-        <v>0.239428</v>
+        <v>0.236031</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B83" t="n" s="0">
-        <v>0.0164301</v>
+        <v>0.0164688</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B84" t="n" s="0">
-        <v>4.30146E-4</v>
+        <v>4.6771E-4</v>
       </c>
     </row>
     <row r="85"/>
     <row r="86">
       <c r="A86" t="s" s="1">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B87" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B88" t="n" s="0">
-        <v>6.36928</v>
+        <v>6.36021</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B89" t="n" s="0">
-        <v>22.0749</v>
+        <v>22.0865</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B90" t="n" s="0">
-        <v>31.6469</v>
+        <v>31.6535</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B91" t="n" s="0">
-        <v>24.6101</v>
+        <v>24.6017</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B92" t="n" s="0">
-        <v>11.4009</v>
+        <v>11.4052</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B93" t="n" s="0">
-        <v>3.26254</v>
+        <v>3.25681</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B94" t="n" s="0">
-        <v>0.572411</v>
+        <v>0.574199</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B95" t="n" s="0">
-        <v>0.0595397</v>
+        <v>0.0583884</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="0">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B96" t="n" s="0">
-        <v>0.00325427</v>
+        <v>0.00348332</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s" s="0">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B97" t="n" s="0">
-        <v>5.93975E-5</v>
+        <v>4.50042E-5</v>
       </c>
     </row>
     <row r="98"/>
     <row r="99">
       <c r="A99" t="s" s="1">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B100" t="s" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B101" t="n" s="0">
-        <v>4.57499</v>
+        <v>4.57396</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B102" t="n" s="0">
-        <v>17.9467</v>
+        <v>17.939</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B103" t="n" s="0">
-        <v>29.5212</v>
+        <v>29.5329</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B104" t="n" s="0">
-        <v>26.7437</v>
+        <v>26.7426</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s" s="0">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B105" t="n" s="0">
-        <v>14.7348</v>
+        <v>14.7346</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s" s="0">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B106" t="n" s="0">
-        <v>5.1487</v>
+        <v>5.14895</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s" s="0">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B107" t="n" s="0">
-        <v>1.15346</v>
+        <v>1.15208</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s" s="0">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B108" t="n" s="0">
-        <v>0.162313</v>
+        <v>0.161098</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s" s="0">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B109" t="n" s="0">
-        <v>0.0134791</v>
+        <v>0.0140774</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s" s="0">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B110" t="n" s="0">
-        <v>6.58836E-4</v>
+        <v>6.93067E-4</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s" s="0">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B111" t="n" s="0">
-        <v>1.44008E-5</v>
+        <v>9.00087E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>